<commit_message>
feat: deploy conversational Excel formula and VBA editing
</commit_message>
<xml_diff>
--- a/public/excel-converter/examples/11_타회사위임장_개인별양식.xlsx
+++ b/public/excel-converter/examples/11_타회사위임장_개인별양식.xlsx
@@ -4,6 +4,9 @@
   <x:sheets>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개인위임장" sheetId="1" r:id="Rfb4973f02ae24912"/>
   </x:sheets>
+  <x:definedNames>
+    <x:definedName name="_xlnm.Print_Area" localSheetId="0">'개인위임장'!$A$1:$F$25</x:definedName>
+  </x:definedNames>
 </x:workbook>
 </file>
 
@@ -283,6 +286,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:pageSetUpPr fitToPage="1"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="17" hidden="0" customWidth="1"/>
@@ -561,5 +567,6 @@
     <x:mergeCell ref="A25:F25"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
chore: checkpoint local work and exclude generated artifacts
</commit_message>
<xml_diff>
--- a/public/excel-converter/examples/11_타회사위임장_개인별양식.xlsx
+++ b/public/excel-converter/examples/11_타회사위임장_개인별양식.xlsx
@@ -4,6 +4,9 @@
   <x:sheets>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개인위임장" sheetId="1" r:id="Rfb4973f02ae24912"/>
   </x:sheets>
+  <x:definedNames>
+    <x:definedName name="_xlnm.Print_Area" localSheetId="0">'개인위임장'!$A$1:$F$25</x:definedName>
+  </x:definedNames>
 </x:workbook>
 </file>
 
@@ -283,6 +286,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:pageSetUpPr fitToPage="1"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="17" hidden="0" customWidth="1"/>
@@ -561,5 +567,6 @@
     <x:mergeCell ref="A25:F25"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
 </x:worksheet>
 </file>
</xml_diff>